<commit_message>
data(nzd): daily refresh 2026-09-21T09:39Z
</commit_message>
<xml_diff>
--- a/logs/nzd/raw/D9.xlsx
+++ b/logs/nzd/raw/D9.xlsx
@@ -50739,6 +50739,78 @@
         <v>129</v>
       </c>
     </row>
+    <row r="911">
+      <c r="A911" s="27">
+        <v>46283</v>
+      </c>
+      <c r="B911" s="16">
+        <v>72538</v>
+      </c>
+      <c r="C911"/>
+      <c r="D911"/>
+      <c r="E911"/>
+      <c r="F911"/>
+      <c r="G911"/>
+      <c r="H911"/>
+      <c r="I911" s="16">
+        <v>3590</v>
+      </c>
+      <c r="J911" s="16">
+        <v>6466</v>
+      </c>
+      <c r="K911" s="16">
+        <v>7555</v>
+      </c>
+      <c r="L911" s="16">
+        <v>6477</v>
+      </c>
+      <c r="M911" s="16">
+        <v>11700</v>
+      </c>
+      <c r="N911" s="16">
+        <v>13191</v>
+      </c>
+      <c r="O911" s="16">
+        <v>3521</v>
+      </c>
+      <c r="P911" s="16">
+        <v>2100</v>
+      </c>
+      <c r="Q911" s="16">
+        <v>5293</v>
+      </c>
+      <c r="R911" s="16">
+        <v>6383</v>
+      </c>
+      <c r="S911" s="16">
+        <v>1993</v>
+      </c>
+      <c r="T911" s="16">
+        <v>1211</v>
+      </c>
+      <c r="U911" s="16">
+        <v>550</v>
+      </c>
+      <c r="V911" s="16">
+        <v>374</v>
+      </c>
+      <c r="W911" s="16">
+        <v>531</v>
+      </c>
+      <c r="X911"/>
+      <c r="Y911" s="16">
+        <v>546</v>
+      </c>
+      <c r="Z911" s="16">
+        <v>412</v>
+      </c>
+      <c r="AA911" s="16">
+        <v>624</v>
+      </c>
+      <c r="AB911" s="16">
+        <v>22</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B5" location="'Series Definitions'!R2C3"/>
@@ -50811,7 +50883,7 @@
         <v>66</v>
       </c>
       <c r="B4" s="27">
-        <v>46279</v>
+        <v>46286</v>
       </c>
     </row>
     <row r="5"/>

</xml_diff>

<commit_message>
data(nzd): daily refresh 2026-10-05T11:13Z
</commit_message>
<xml_diff>
--- a/logs/nzd/raw/D9.xlsx
+++ b/logs/nzd/raw/D9.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\rbnz\dfs\homedrives2\wangcl\Desktop\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{47674C76-D4C3-49DD-850F-0DA69DFBF977}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{4DD8EF11-E689-4F4B-A841-189C155359B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2280" yWindow="2280" windowWidth="14400" windowHeight="8170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -696,7 +696,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AB912"/>
+  <dimension ref="A1:AB913"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13.6328125" customWidth="1" collapsed="1"/>
@@ -36998,6 +36998,71 @@
       </c>
       <c r="AB912" s="7">
         <v>75</v>
+      </c>
+    </row>
+    <row r="913" spans="1:28" x14ac:dyDescent="0.35">
+      <c r="A913" s="8">
+        <v>46297</v>
+      </c>
+      <c r="B913" s="7">
+        <v>86750</v>
+      </c>
+      <c r="I913" s="7">
+        <v>2082</v>
+      </c>
+      <c r="J913" s="7">
+        <v>6583</v>
+      </c>
+      <c r="K913" s="7">
+        <v>7034</v>
+      </c>
+      <c r="L913" s="7">
+        <v>10181</v>
+      </c>
+      <c r="M913" s="7">
+        <v>17347</v>
+      </c>
+      <c r="N913" s="7">
+        <v>7939</v>
+      </c>
+      <c r="O913" s="7">
+        <v>4494</v>
+      </c>
+      <c r="P913" s="7">
+        <v>3959</v>
+      </c>
+      <c r="Q913" s="7">
+        <v>8175</v>
+      </c>
+      <c r="R913" s="7">
+        <v>8094</v>
+      </c>
+      <c r="S913" s="7">
+        <v>4603</v>
+      </c>
+      <c r="T913" s="7">
+        <v>2349</v>
+      </c>
+      <c r="U913" s="7">
+        <v>599</v>
+      </c>
+      <c r="V913" s="7">
+        <v>1055</v>
+      </c>
+      <c r="W913" s="7">
+        <v>573</v>
+      </c>
+      <c r="Y913" s="7">
+        <v>402</v>
+      </c>
+      <c r="Z913" s="7">
+        <v>486</v>
+      </c>
+      <c r="AA913" s="7">
+        <v>735</v>
+      </c>
+      <c r="AB913" s="7">
+        <v>63</v>
       </c>
     </row>
   </sheetData>
@@ -37076,7 +37141,7 @@
         <v>66</v>
       </c>
       <c r="B4" s="8">
-        <v>46293</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
data(nzd): daily refresh 2026-10-12T11:42Z
</commit_message>
<xml_diff>
--- a/logs/nzd/raw/D9.xlsx
+++ b/logs/nzd/raw/D9.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\rbnz\dfs\homedrives2\wangcl\Desktop\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{4DD8EF11-E689-4F4B-A841-189C155359B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{1D5E9077-1890-48B4-A003-E3CAB83764DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10080" yWindow="2730" windowWidth="25270" windowHeight="15850" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -696,7 +696,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AB913"/>
+  <dimension ref="A1:AB914"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13.6328125" customWidth="1" collapsed="1"/>
@@ -37063,6 +37063,71 @@
       </c>
       <c r="AB913" s="7">
         <v>63</v>
+      </c>
+    </row>
+    <row r="914" spans="1:28" x14ac:dyDescent="0.35">
+      <c r="A914" s="8">
+        <v>46304</v>
+      </c>
+      <c r="B914" s="7">
+        <v>77168</v>
+      </c>
+      <c r="I914" s="7">
+        <v>1396</v>
+      </c>
+      <c r="J914" s="7">
+        <v>6819</v>
+      </c>
+      <c r="K914" s="7">
+        <v>5185</v>
+      </c>
+      <c r="L914" s="7">
+        <v>8917</v>
+      </c>
+      <c r="M914" s="7">
+        <v>12475</v>
+      </c>
+      <c r="N914" s="7">
+        <v>7656</v>
+      </c>
+      <c r="O914" s="7">
+        <v>5372</v>
+      </c>
+      <c r="P914" s="7">
+        <v>2999</v>
+      </c>
+      <c r="Q914" s="7">
+        <v>8648</v>
+      </c>
+      <c r="R914" s="7">
+        <v>5398</v>
+      </c>
+      <c r="S914" s="7">
+        <v>3782</v>
+      </c>
+      <c r="T914" s="7">
+        <v>4516</v>
+      </c>
+      <c r="U914" s="7">
+        <v>847</v>
+      </c>
+      <c r="V914" s="7">
+        <v>1280</v>
+      </c>
+      <c r="W914" s="7">
+        <v>394</v>
+      </c>
+      <c r="Y914" s="7">
+        <v>162</v>
+      </c>
+      <c r="Z914" s="7">
+        <v>482</v>
+      </c>
+      <c r="AA914" s="7">
+        <v>655</v>
+      </c>
+      <c r="AB914" s="7">
+        <v>184</v>
       </c>
     </row>
   </sheetData>
@@ -37141,7 +37206,7 @@
         <v>66</v>
       </c>
       <c r="B4" s="8">
-        <v>46300</v>
+        <v>46307</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">

</xml_diff>